<commit_message>
Update latest job list
</commit_message>
<xml_diff>
--- a/jobs_latest.xlsx
+++ b/jobs_latest.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Latest Jobs'!$A$1:$M$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Latest Jobs'!$A$1:$M$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M106"/>
+  <dimension ref="A1:M99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9389,492 +9389,9 @@
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>expleo-jobs-gb-en</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>Automotive Cybersecurity Engineer</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>Preston, LNH, GB</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
-      <c r="H100" s="2" t="inlineStr"/>
-      <c r="I100" s="2" t="inlineStr">
-        <is>
-          <t>FULL_TIME</t>
-        </is>
-      </c>
-      <c r="J100" s="2" t="inlineStr">
-        <is>
-          <t>icims</t>
-        </is>
-      </c>
-      <c r="K100" s="3" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="L100" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M100" s="2" t="inlineStr">
-        <is>
-          <t>As part of the Expleo Automotive &amp; Transportation Cybersecurity team, you will report to the Solution Architect / Head of Function and support client projects. Within the Automotive &amp; Transportation Cybersecurity Practice, you will be part of a dynamic and passionate team. You will work on a complex and captivating projects integrating the latest technological solutions and trends.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="B101" s="2" t="inlineStr">
-        <is>
-          <t>Motorola Solutions</t>
-        </is>
-      </c>
-      <c r="C101" s="2" t="inlineStr">
-        <is>
-          <t>Senior Software Cybersecurity Engineer</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>Uxbridge, United Kingdom</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="F101" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G101" s="2" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
-      <c r="H101" s="2" t="inlineStr"/>
-      <c r="I101" s="2" t="inlineStr">
-        <is>
-          <t>FULL_TIME</t>
-        </is>
-      </c>
-      <c r="J101" s="2" t="inlineStr">
-        <is>
-          <t>welcometothejungle</t>
-        </is>
-      </c>
-      <c r="K101" s="3" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="L101" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M101" s="2" t="inlineStr">
-        <is>
-          <t>Join our team as a Senior Software Cybersecurity Engineer. In this role, you will analyze software designs and implementations to identify and remediate security vulnerabilities across the software development lifecycle (SDLC). You will perform threat modeling, risk assessments, audits, and architecture reviews, focusing on cloud and container environments. You will also manage key management and IAM controls, support engineering teams by defining security requirements, and perform security code reviews. Additionally, you will drive vulnerability management, support product security incident response, and monitor emerging threats to ensure compliance with standards.
-- Analyser les conceptions et les mises en œuvre logicielles pour identifier et remédier aux vulnérabilités de sécurité tout au long du cycle de vie du développement logiciel (SDLC).
-- Effectuer des tests de sécurité, déployer et gérer des outils de sécurité automatisés dans les pipelines CI/CD, et recommander des améliorations aux outils de sécurité existants.
-- Gérer la gestion des vulnérabilités, en mettant l'accent sur Kubernetes (K8s) et les images de conteneurs, et communiquer les problèmes de sécurité aux parties prenantes.
- - Software Engineering: Hands-on development experience, specifically in Go and C#
-- Leadership: Proven track record in leading process change, mentoring on secure-by-design principles, and driving continuous improvement
-- Experience &amp; Education: 7+ years in Security/Application Engineering; Bachelor’s degree in Computer Science, Information Security, or a related field
-- AppSec &amp; DevSecOps: Deep understanding of threat modeling (STRIDE, PASTA), IAM, cryptography, web/network protocols (HTTP, REST, TLS, TCP/IP), and integrating security tooling (SCA, SAST, DAST) into CI/CD pipelines
-- Cloud &amp; Container Security: Strong knowledge of orchestration (AWS, Azure, GCP, Docker, Kubernetes) and container image vulnerability lifecycles
-- Standards &amp; Frameworks: Knowledge of NIST, ISO 27001, CIS, and OWASP (ASVS/Testing Guides)
-- Advanced Technical Skills: Deep vulnerability research, exploit R&amp;D, manual pentesting (cloud/web/embedded/mobile), SIEM/logging platforms (Splunk, OSQuery), AI/ML security, and distributed systems
-- Education &amp; Certifications: Master’s degree preferred; Cloud/Security certifications (CCSP, CCAK, AWS Security Specialty, OSCP, CISSP, SANS/GIAC)
-- Soft Skills: Strong communication across technical and non-technical groups, calm under pressure, and experience in high-growth SaaS environments</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="inlineStr">
-        <is>
-          <t>dLocal</t>
-        </is>
-      </c>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>Principal Security Engineer (Identity &amp; Access)</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>Madrid, Spain</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="F102" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G102" s="2" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
-      <c r="H102" s="2" t="inlineStr"/>
-      <c r="I102" s="2" t="inlineStr">
-        <is>
-          <t>FULL_TIME</t>
-        </is>
-      </c>
-      <c r="J102" s="2" t="inlineStr">
-        <is>
-          <t>welcometothejungle</t>
-        </is>
-      </c>
-      <c r="K102" s="3" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="L102" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M102" s="2" t="inlineStr">
-        <is>
-          <t>Join our rapidly evolving fintech company as a Principal Security Engineer specializing in Identity &amp; Access. In this hands-on role, you will engineer a highly automated identity lifecycle, design and scale our authentication and authorization foundations, lead identity integration strategies for mergers and acquisitions, and codify governance. You will collaborate with various teams across the organization and have a strong impact on our identity transformation.
-- Conduire l'évolution de l'identité de l'entreprise en concevant et en mettant en œuvre des solutions d'automatisation pour le cycle de vie des identités.
-- Diriger la stratégie d'intégration des identités pour les fusions, acquisitions et initiatives de transformation d'entreprise.
-- Collaborer avec les équipes interfonctionnelles pour gouverner l'accès à travers l'entreprise et le cloud.
- - Pragmatic Operator Mindset: You understand that security cannot kill velocity. You know how to find the critical balance between enforcing strict, least-privilege security and maintaining high usability for the business
-- Disciplined Multi-Threading: You are ruthlessly organized, capable of driving an enterprise identity strategy while simultaneously troubleshooting an immediate, ground-level access escalation
-- Deep IGA &amp; Protocol Expertise: You possess solid, hands-on experience with modern workforce identity systems, lifecycle processes (JML, SoD, Certifications), protocols (SAML, OIDC, OAuth2, SCIM), RBAC/ABAC models, and enterprise identity platforms (e.g., SailPoint, Saviynt, Okta)
-- Force Multiplier: You elevate the engineers around you. You bring strong mentoring, leadership, and documentation capabilities, ensuring that the systems you design are highly scalable, well-understood, and easily maintained by the wider organization
-- Track Record Over Tenure: We do not care about arbitrary "years of experience." We care about outcomes. You must have a proven track record of designing, building, or scaling Identity and Access programs in fast-paced, complex environments
-- Resilient Problem Solver: You don't get stuck. Where others see a messy legacy setup, you see an exciting puzzle. You don't get paralyzed or frustrated by organizational friction; you thrive on using the latest technologies and original thinking to solve long-standing identity problems
-- Relevant industry certifications demonstrating your dedication to the identity domain
-- Familiarity with machine identity governance, secrets management, and API access
-- Experience navigating the identity and access requirements of highly regulated environments (PCI-DSS, SOX, SOC 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="B103" s="2" t="inlineStr">
-        <is>
-          <t>brightvisiontechnologies</t>
-        </is>
-      </c>
-      <c r="C103" s="2" t="inlineStr">
-        <is>
-          <t>Software Security Engineer</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="E103" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="F103" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G103" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H103" s="2" t="inlineStr">
-        <is>
-          <t>USD 145,000–165,000 / year</t>
-        </is>
-      </c>
-      <c r="I103" s="2" t="inlineStr">
-        <is>
-          <t>FULL_TIME</t>
-        </is>
-      </c>
-      <c r="J103" s="2" t="inlineStr">
-        <is>
-          <t>jazzhr</t>
-        </is>
-      </c>
-      <c r="K103" s="3" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="L103" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M103" s="2" t="inlineStr">
-        <is>
-          <t>Bright Vision Technologies is a technology consulting and software development company delivering cloud, AI, data, and enterprise solutions across the United States. This is a fantastic opportunity to join an established and well-respected organization offering tremendous career growth potential. Job Title: Software Security Engineer Location: 100% Remote (U.S.) Position Type: Full-time, Direct W2 Salary Range: $145,000–$165,000 Annually Experience Required: 6+ years Sponsorship: U.S. Citizens, Green Card Holders, EAD Holders, and H-1B transfer candidates are encouraged to apply. We are unable to sponsor new H-1B visa petitions for this position. Job Summary: We are looking for an Software Security Engineer to embed security throughout the software development lifecycle, partnering with engineering teams to design secure systems, identify vulnerabilities, and reduce risk across our application portfolio. The role blends hands-on offensive and defensive skills with strong communication and collaboration, helping development teams build secure software efficiently rather than slowing them down. The ideal candidate brings deep technical security expertise, strong software engineering fundamentals, and a track record of shipping security improvements that meaningfully reduce risk in production. Required Qualifications Bachelor’s degree in Computer Science, Cybersecurity, or a related field. Five or more years of application security or security engineering experience. Strong understanding of OWASP Top 10, common vulnerability classes, and modern exploit patterns. Hands-on experience performing code review across at least two major languages. Deep familiarity with SAST, DAST, SCA, and CI/CD-integrated security tooling. Strong understanding of authentication, authorization, and cryptographic primitives. Experience with cloud security and modern infrastructure controls. Strong communication skills with technical and non-technical audiences. Proficiency in at least one programming language for tooling and automation. Experience working closely with engineering teams in an Agile environment. Preferred Qualifications Industry certifications such as OSCP, OSCE, GWAPT, or CISSP. Experience with offensive security tooling and red-team operations. Bug bounty experience, public CVEs, or open-source security contributions. Familiarity with AI/LLM application security considerations. Exposure to regulated industries with strict compliance requirements. How to Apply Would you like to know more about this opportunity? For immediate consideration, please send your resume to or contact us at (908)676-4399. Learn more about Bright Vision Technologies at . Bright Vision Technologies is an Equal Opportunity Employer Equal Employment Opportunity (EEO) Statement Bright Vision Technologies (BV Teck) is committed to equal employment opportunity (EEO) for all employees and applicants without regard to race, color, religion, sex, sexual orientation, gender identity or expression, national origin, age, genetic information, disability, veteran status, or any other protected status as defined by applicable federal, state, or local laws. This commitment extends to all aspects of employment, including recruitment, hiring, training, compensation, promotion, transfer, leaves of absence, termination, layoffs, and recall. BV Teck expressly prohibits any form of workplace harassment or discrimination. Any improper interference with employees' ability to perform their job duties may result in disciplinary action up to and including termination of employment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr">
-        <is>
-          <t>careers.roche.com</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>Cybersecurity Engineer -  Monitoring &amp; Incident Response</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>Madrid, Spain</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G104" s="2" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
-      <c r="H104" s="2" t="inlineStr"/>
-      <c r="I104" s="2" t="inlineStr"/>
-      <c r="J104" s="2" t="inlineStr">
-        <is>
-          <t>phenom</t>
-        </is>
-      </c>
-      <c r="K104" s="3" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="L104" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M104" s="2" t="inlineStr">
-        <is>
-          <t>Become part of our team as a Cybersecurity Engineer in Monitoring &amp; Incident Response, where you will protect Roche’s global networks and users from evolving threats. You will monitor security information, respond to incidents, and support continuous improvement. Ideal candidates bring significant experience in information security and a strong background in SOC/CERT/CSIRT environments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="B105" s="2" t="inlineStr">
-        <is>
-          <t>careers.statestreet.com</t>
-        </is>
-      </c>
-      <c r="C105" s="2" t="inlineStr">
-        <is>
-          <t>Cybersecurity Automation Engineer ,Assistant Vice President</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>Kilkenny, Kilkenny, Ireland</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>IE</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G105" s="2" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
-      <c r="H105" s="2" t="inlineStr"/>
-      <c r="I105" s="2" t="inlineStr"/>
-      <c r="J105" s="2" t="inlineStr">
-        <is>
-          <t>phenom</t>
-        </is>
-      </c>
-      <c r="K105" s="3" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="L105" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M105" s="2" t="inlineStr">
-        <is>
-          <t>We are looking for a Cybersecurity Automation Engineer, Assistant Vice President, to identify and implement automation opportunities within our SOC. You will collaborate with analysts to enhance incident response workflows and develop user stories. Ideal candidates have experience in cybersecurity and strong programming skills.</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B106" s="2" t="inlineStr">
-        <is>
-          <t>Neon</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>Nuclear Security Engineer</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G106" s="2" t="inlineStr">
-        <is>
-          <t>Not mentioned</t>
-        </is>
-      </c>
-      <c r="H106" s="2" t="inlineStr">
-        <is>
-          <t>$65–75/per-task</t>
-        </is>
-      </c>
-      <c r="I106" s="2" t="inlineStr">
-        <is>
-          <t>CONTRACT</t>
-        </is>
-      </c>
-      <c r="J106" s="2" t="inlineStr">
-        <is>
-          <t>mercor</t>
-        </is>
-      </c>
-      <c r="K106" s="3" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="L106" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M106" s="2" t="inlineStr">
-        <is>
-          <t>## About the work
-Mercor is assembling a panel of nuclear materials and safeguards experts to red-team frontier AI models. The goal is to test whether a model can correctly judge the misuse potential of a technical request — answering legitimate questions fully while refusing genuinely dangerous ones.
-You will:
-- Write challenging single-turn prompts in your domain, labelled across three levels: benign, dual-use, and adversarial.
-- Evaluate the responses that come back against a defined policy standard, and judge whether each was handled correctly.
-- Write the reference answer — what a correct response looks like, and the technical reasoning for why.
-This domain lives on the dual-use line more than most. The same material-balance calculation that closes an inspector's account can be used to hide what is missing from it; the same protection assessment that hardens a facility maps its weaknesses. A model that refuses a routine material-accounting question is failing as badly as one that answers a question it shouldn't. Drawing that line reliably is why we need practitioners rather than generalists.
-## Background we're looking for
-We're looking for people who have been responsible for keeping nuclear material where it belongs — material control and accountability, physical protection, and the assessments that test both. What matters most is being able to tell a routine professional question from one that's fishing for something else: the same vulnerability assessment that closes a gap also describes it. You will be writing prompts that sit exactly on that line, then judging whether the model held it.
-Examples of relevant backgrounds (ideally with red-teaming experience):
-- Material control and accountability (MC&amp;A) programme design, operation or assessment at a national laboratory or licensee
-- Physical protection system engineering — sensors, barriers, delay, response force, performance testing
-- Vulnerability assessment and adversary path analysis for nuclear facilities
-- Insider threat and human reliability programme work
-- Nuclear security policy, training or international assistance programmes
-## What this role demands beyond technical depth
-This is writing-intensive work. Every judgment you make needs a written rationale that a non-specialist can follow. Prior technical writing, published research, or expert witness experience is a strong signal; please include a sample or link. You will also be reading and writing about misuse scenarios in your field for sustained periods. We brief experts on this in advance, and you can pause or step away at any point without penalty.
-## Before you apply
-Your work here will not involve, and must not draw on, classified or export-controlled information, or anything covered by an NDA or prepublication review obligation. If you hold such obligations you may still be a good fit; tell us in your application and we will scope the work accordingly.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M106"/>
-  <conditionalFormatting sqref="A2:M106">
+  <autoFilter ref="A1:M99"/>
+  <conditionalFormatting sqref="A2:M99">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="New"</formula>
     </cfRule>
@@ -9889,7 +9406,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="L2 L3 L4 L5 L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L45 L46 L47 L48 L49 L50 L51 L52 L53 L54 L55 L56 L57 L58 L59 L60 L61 L62 L63 L64 L65 L66 L67 L68 L69 L70 L71 L72 L73 L74 L75 L76 L77 L78 L79 L80 L81 L82 L83 L84 L85 L86 L87 L88 L89 L90 L91 L92 L93 L94 L95 L96 L97 L98 L99 L100 L101 L102 L103 L104 L105 L106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Status" error="Please select a valid status" type="list">
+    <dataValidation sqref="L2 L3 L4 L5 L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L45 L46 L47 L48 L49 L50 L51 L52 L53 L54 L55 L56 L57 L58 L59 L60 L61 L62 L63 L64 L65 L66 L67 L68 L69 L70 L71 L72 L73 L74 L75 L76 L77 L78 L79 L80 L81 L82 L83 L84 L85 L86 L87 L88 L89 L90 L91 L92 L93 L94 L95 L96 L97 L98 L99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Status" error="Please select a valid status" type="list">
       <formula1>"New,Opened,Applied,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9992,13 +9509,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K100" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId105"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>